<commit_message>
feat(F-NAR-009): DIF + deux ramifiées AUT-015/016
Ouvertures du monde, pas de constat sec. Texte seulement.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-06.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-06.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Adèle répète, Estelle observe</t>
+          <t>Raphaël répète, Aniss observe</t>
         </is>
       </c>
     </row>
@@ -602,6 +602,11 @@
           <t>secondary_lessons</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DIF.BES.002</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -830,6 +835,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Raphaël veut les cubes jaunes. Aniss a besoin de calme. Raphaël répète. Aniss observe d'abord.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Adèle arrive en classe. Papa est à la porte. Un jeu commence. On pose un cube. Puis on attend. Estelle reste près du mur. Elle a besoin de calme. Adèle va vers Estelle. Adèle va répéter la règle. Un cube, puis on attend. Estelle écoute. Elle va observer d'abord. Observer d'abord, c'est possible. Adèle joue. Estelle regarde. On peut répéter. On peut observer d'abord. Plus tard, Estelle s'assoit. Elle pose un cube. C'est assez.</t>
+          <t>La vitre de la classe est embuée. Des gouttes glissent tout doux. Les manteaux gouttent dans le couloir. Ça sent le savon. Un panier rond attend près du tapis. Dedans, des cubes jaunes. Papa accroche le petit manteau bleu. Tu vois le jardin, Raphaël ? Oui, maman. Maman essuie un coin de vitre. Les arbres sont tout mouillés. On rentre au calme. Le tapis est déjà là. En ce moment, Raphaël s'assoit. Le tapis rouge est doux. Ses genoux sentent la laine. Aniss arrive tout doux. Aniss s'arrête près du mur. Il a besoin de calme. Maman, on joue ? Oui. On pose un cube. Puis on attend. Raphaël prend un cube jaune. Le cube est lisse et chaud. Il va vers Aniss. Il parle tout bas. Un cube. Puis on attend. Aniss écoute. Il regarde le panier. On peut répéter. On peut observer d'abord. Observer d'abord, c'est possible. Raphaël pose son cube. Il attend. Aniss regarde. Ses mains restent sur ses genoux. Un cube touche un autre cube. Ça fait un petit bruit. Tu as entendu le cube ? Oui, papa. Raphaël pose un autre cube. Jaune encore. Aniss avance un pied. Puis il s'assoit au bord. Il observe d'abord. Plus tard, il pose un cube. Tout doux. C'est assez. Tu as répété, Raphaël. Bravo. Tu as fait du bon travail. Aniss a observé d'abord. Oui. Il a pu observer d'abord.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,13 +1329,69 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Adèle arrive en classe. Papa est à la porte. Un jeu commence. On pose un cube. Puis on attend. Estelle reste près du mur. Elle a besoin de calme. Adèle va vers Estelle. Adèle va répéter la règle.
-enfant-f|Un cube, puis on attend.
-narrateur|Estelle écoute. Elle va observer d'abord. Observer d'abord, c'est possible. Adèle joue. Estelle regarde.
-papa|On peut répéter. On peut observer d'abord. Plus tard, Estelle s'assoit. Elle pose un cube. C'est assez.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+          <t>narrateur|La vitre de la classe est embuée.
+narrateur|Des gouttes glissent tout doux.
+narrateur|Les manteaux gouttent dans le couloir.
+narrateur|Ça sent le savon.
+narrateur|Un panier rond attend près du tapis.
+narrateur|Dedans, des cubes jaunes.
+narrateur|Papa accroche le petit manteau bleu.
+maman|Tu vois le jardin, Raphaël ?
+enfant-m|Oui, maman.
+narrateur|Maman essuie un coin de vitre.
+maman|Les arbres sont tout mouillés.
+papa|On rentre au calme.
+papa|Le tapis est déjà là.
+narrateur|En ce moment, Raphaël s'assoit.
+narrateur|Le tapis rouge est doux.
+narrateur|Ses genoux sentent la laine.
+narrateur|Aniss arrive tout doux.
+narrateur|Aniss s'arrête près du mur.
+narrateur|Il a besoin de calme.
+enfant-m|Maman, on joue ?
+maman|Oui.
+maman|On pose un cube.
+maman|Puis on attend.
+narrateur|Raphaël prend un cube jaune.
+narrateur|Le cube est lisse et chaud.
+narrateur|Il va vers Aniss.
+narrateur|Il parle tout bas.
+enfant-m|Un cube.
+enfant-m|Puis on attend.
+narrateur|Aniss écoute.
+narrateur|Il regarde le panier.
+papa|On peut répéter.
+papa|On peut observer d'abord.
+maman|Observer d'abord, c'est possible.
+narrateur|Raphaël pose son cube.
+narrateur|Il attend.
+narrateur|Aniss regarde.
+narrateur|Ses mains restent sur ses genoux.
+narrateur|Un cube touche un autre cube.
+narrateur|Ça fait un petit bruit.
+papa|Tu as entendu le cube ?
+enfant-m|Oui, papa.
+narrateur|Raphaël pose un autre cube.
+narrateur|Jaune encore.
+narrateur|Aniss avance un pied.
+narrateur|Puis il s'assoit au bord.
+narrateur|Il observe d'abord.
+narrateur|Plus tard, il pose un cube.
+narrateur|Tout doux.
+maman|C'est assez.
+papa|Tu as répété, Raphaël.
+papa|Bravo.
+maman|Tu as fait du bon travail.
+enfant-m|Aniss a observé d'abord.
+maman|Oui.
+maman|Il a pu observer d'abord.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>pluie,manteaux</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1343,7 +1416,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Estelle a besoin de calme. Que peut-on faire ?</t>
+          <t>Aniss a besoin de calme. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1499,7 +1572,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Estelle a besoin de calme. Que peut-on faire ?</t>
+          <t>narrateur|Aniss a besoin de calme.
+narrateur|Que peut-on faire ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1527,7 +1601,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Adèle a su répéter. Estelle a pu observer d'abord. Le jeu a continué.</t>
+          <t>Raphaël a su répéter. Aniss a pu observer d'abord. Le jeu a continué, tout doux. Le tapis reste rouge et chaud. Tu as laissé le temps ? Oui, papa. Bravo. Observer d'abord, c'est bien. Aniss touche encore un cube. Il le pose près des autres. Raphaël attend. C'est du bon travail.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1671,7 +1745,18 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Adèle a su répéter. Estelle a pu observer d'abord. Le jeu a continué.</t>
+          <t>narrateur|Raphaël a su répéter.
+narrateur|Aniss a pu observer d'abord.
+narrateur|Le jeu a continué, tout doux.
+narrateur|Le tapis reste rouge et chaud.
+papa|Tu as laissé le temps ?
+enfant-m|Oui, papa.
+maman|Bravo.
+maman|Observer d'abord, c'est bien.
+narrateur|Aniss touche encore un cube.
+narrateur|Il le pose près des autres.
+narrateur|Raphaël attend.
+papa|C'est du bon travail.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1699,7 +1784,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa reprend Adèle. Estelle range un cube.</t>
+          <t>On range les cubes ? Oui. Raphaël met un cube dans le panier. Aniss met un cube aussi. Le panier redevient lourd. Tu as fini de ranger tes cubes ? Oui, papa. Bravo, Raphaël. Merci, Aniss. Papa tend la main. Le couloir sent encore le savon. Les manteaux sont un peu secs.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1835,7 +1920,18 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa reprend Adèle. Estelle range un cube.</t>
+          <t>maman|On range les cubes ?
+enfant-m|Oui.
+narrateur|Raphaël met un cube dans le panier.
+narrateur|Aniss met un cube aussi.
+narrateur|Le panier redevient lourd.
+papa|Tu as fini de ranger tes cubes ?
+enfant-m|Oui, papa.
+papa|Bravo, Raphaël.
+maman|Merci, Aniss.
+narrateur|Papa tend la main.
+narrateur|Le couloir sent encore le savon.
+narrateur|Les manteaux sont un peu secs.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1863,7 +1959,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>On a répété. Aniss a observé d'abord. Bravo. Tu as fait du bon travail. Les cubes jaunes dorment. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2003,7 +2099,12 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-m|On a répété.
+enfant-m|Aniss a observé d'abord.
+maman|Bravo.
+papa|Tu as fait du bon travail.
+narrateur|Les cubes jaunes dorment.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2025,7 +2126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2063,6 +2164,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-008): 16 ATOM de plus (BES / PAR)
Histoires, pas des listes.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-06.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Raphaël répète, Aniss observe</t>
+          <t>Le train sous la table</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut les cubes jaunes. Aniss a besoin de calme. Raphaël répète. Aniss observe d'abord.</t>
+          <t>Raphaël veut que son train de bois passe sous la table jusqu'à la chaise. Aniss reste près du buffet. Raphaël répète : un wagon, puis on attend. Aniss observe d'abord, puis pose le wagon rouge. Le train arrive.</t>
         </is>
       </c>
     </row>
@@ -1189,12 +1189,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La vitre de la classe est embuée. Des gouttes glissent tout doux. Les manteaux gouttent dans le couloir. Ça sent le savon. Un panier rond attend près du tapis. Dedans, des cubes jaunes. Papa accroche le petit manteau bleu. Tu vois le jardin, Raphaël ? Oui, maman. Maman essuie un coin de vitre. Les arbres sont tout mouillés. On rentre au calme. Le tapis est déjà là. En ce moment, Raphaël s'assoit. Le tapis rouge est doux. Ses genoux sentent la laine. Aniss arrive tout doux. Aniss s'arrête près du mur. Il a besoin de calme. Maman, on joue ? Oui. On pose un cube. Puis on attend. Raphaël prend un cube jaune. Le cube est lisse et chaud. Il va vers Aniss. Il parle tout bas. Un cube. Puis on attend. Aniss écoute. Il regarde le panier. On peut répéter. On peut observer d'abord. Observer d'abord, c'est possible. Raphaël pose son cube. Il attend. Aniss regarde. Ses mains restent sur ses genoux. Un cube touche un autre cube. Ça fait un petit bruit. Tu as entendu le cube ? Oui, papa. Raphaël pose un autre cube. Jaune encore. Aniss avance un pied. Puis il s'assoit au bord. Il observe d'abord. Plus tard, il pose un cube. Tout doux. C'est assez. Tu as répété, Raphaël. Bravo. Tu as fait du bon travail. Aniss a observé d'abord. Oui. Il a pu observer d'abord. Une goutte glisse encore sur la vitre. Elle va tout droit, puis elle tourne. Tu la vois, Raphaël ? Oui. Raphaël attend encore un peu. Aniss pose sa main près du panier. Il prend un cube jaune. Il le tourne. Le cube est lisse. Tu as répété la règle ? Un cube. Puis on attend. Bravo. Le tapis rouge reste chaud. Le savon sent encore dans le couloir.</t>
+          <t>La confiture d'abricot brille dans le pot. Elle est orange et un peu épaisse. Le pain grillé sent encore le four. Une miette colle à la nappe. La nappe a des carreaux rouges. Papa essuie la cuillère de bois. Raphaël, tu veux de la confiture ? Oui, papa. Un peu, s'il te plaît. Maman ouvre le tiroir du bas. Dedans, le train de bois attend. Les wagons sont lisses et froids. Tu as vu le train, Raphaël ? Oui. Il va sous la table. Jusqu'à la chaise ? Oui. Le wagon rouge aussi. En ce moment, Raphaël s'assoit. Le carrelage est un peu froid. Il pose un wagon brun. Ça fait un petit clic. Tu as entendu le clic ? Oui, papa. Maman ouvre la porte. Aniss arrive tout doux. Il reste près du buffet. Ses mains touchent le bois. Il a besoin de calme. Aniss. Tu viens ? Aniss ne vient pas encore. Le wagon rouge est pour lui. Raphaël regarde papa. On peut répéter, tout doux. On peut observer d'abord. D'accord. Le wagon rouge attend par terre. Il est lisse et froid. Tu parles tout bas, d'accord ? D'accord, papa. Une miette est sur le wagon. Tu as vu la miette ? Oui. Raphaël souffle. La miette part. Le train peut avancer un peu. Raphaël pousse le wagon brun. Aniss regarde, près du buffet. Ses pieds restent au même endroit.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Adèle arrive en classe. Papa est à la porte. Un jeu commence. On pose un cube. Puis on attend. Estelle reste près du mur. Elle a besoin de calme. Adèle va vers Estelle. Adèle va &lt;emphasis level="moderate"&gt;répéter&lt;/emphasis&gt; la règle. Adèle dit : un cube, puis on attend. Estelle écoute. Elle va observer d'abord. Observer d'abord, c'est possible. Adèle joue. Estelle regarde. Papa dit : on peut répéter. On peut observer d'abord. Plus tard, Estelle s'assoit. Elle pose un cube. C'est assez.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>La confiture d'abricot brille dans le pot. Elle est orange et un peu épaisse. Le pain grillé sent encore le four. Une miette colle à la nappe. La nappe a des carreaux rouges. Papa essuie la cuillère de bois. Raphaël, tu veux de la confiture ? Oui, papa. Un peu, s'il te plaît. Maman ouvre le tiroir du bas. Dedans, le train de bois attend. Les wagons sont lisses et froids. Tu as vu le train, Raphaël ? Oui. Il va sous la table. Jusqu'à la chaise ? Oui. Le wagon rouge aussi. En ce moment, Raphaël s'assoit. Le carrelage est un peu froid. Il pose un wagon brun. Ça fait un petit clic. Tu as entendu le clic ? Oui, papa. Maman ouvre la porte. Aniss arrive tout doux. Il reste près du buffet. Ses mains touchent le bois. Il a besoin de calme. Aniss. Tu viens ? Aniss ne vient pas encore. Le wagon rouge est pour lui. Raphaël regarde papa. On peut répéter, tout doux. On peut observer d'abord. D'accord. Le wagon rouge attend par terre. Il est lisse et froid. Tu parles tout bas, d'accord ? D'accord, papa. Une miette est sur le wagon. Tu as vu la miette ? Oui. Raphaël souffle. La miette part. Le train peut avancer un peu. Raphaël pousse le wagon brun. Aniss regarde, près du buffet. Ses pieds restent au même endroit.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
         <v>0.86</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1329,82 +1329,61 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La vitre de la classe est embuée.
-narrateur|Des gouttes glissent tout doux.
-narrateur|Les manteaux gouttent dans le couloir.
-narrateur|Ça sent le savon.
-narrateur|Un panier rond attend près du tapis.
-narrateur|Dedans, des cubes jaunes.
-narrateur|Papa accroche le petit manteau bleu.
-maman|Tu vois le jardin, Raphaël ?
-enfant-m|Oui, maman.
-narrateur|Maman essuie un coin de vitre.
-maman|Les arbres sont tout mouillés.
-papa|On rentre au calme.
-papa|Le tapis est déjà là.
+          <t>narrateur|La confiture d'abricot brille dans le pot.
+narrateur|Elle est orange et un peu épaisse.
+narrateur|Le pain grillé sent encore le four.
+narrateur|Une miette colle à la nappe.
+narrateur|La nappe a des carreaux rouges.
+narrateur|Papa essuie la cuillère de bois.
+papa|Raphaël, tu veux de la confiture ?
+enfant-m|Oui, papa.
+enfant-m|Un peu, s'il te plaît.
+narrateur|Maman ouvre le tiroir du bas.
+narrateur|Dedans, le train de bois attend.
+narrateur|Les wagons sont lisses et froids.
+maman|Tu as vu le train, Raphaël ?
+enfant-m|Oui.
+enfant-m|Il va sous la table.
+maman|Jusqu'à la chaise ?
+enfant-m|Oui.
+enfant-m|Le wagon rouge aussi.
 narrateur|En ce moment, Raphaël s'assoit.
-narrateur|Le tapis rouge est doux.
-narrateur|Ses genoux sentent la laine.
+narrateur|Le carrelage est un peu froid.
+narrateur|Il pose un wagon brun.
+narrateur|Ça fait un petit clic.
+papa|Tu as entendu le clic ?
+enfant-m|Oui, papa.
+narrateur|Maman ouvre la porte.
 narrateur|Aniss arrive tout doux.
-narrateur|Aniss s'arrête près du mur.
+narrateur|Il reste près du buffet.
+narrateur|Ses mains touchent le bois.
 narrateur|Il a besoin de calme.
-enfant-m|Maman, on joue ?
-maman|Oui.
-maman|On pose un cube.
-maman|Puis on attend.
-narrateur|Raphaël prend un cube jaune.
-narrateur|Le cube est lisse et chaud.
-narrateur|Il va vers Aniss.
-narrateur|Il parle tout bas.
-enfant-m|Un cube.
-enfant-m|Puis on attend.
-narrateur|Aniss écoute.
-narrateur|Il regarde le panier.
-papa|On peut répéter.
-papa|On peut observer d'abord.
-maman|Observer d'abord, c'est possible.
-narrateur|Raphaël pose son cube.
-narrateur|Il attend.
-narrateur|Aniss regarde.
-narrateur|Ses mains restent sur ses genoux.
-narrateur|Un cube touche un autre cube.
-narrateur|Ça fait un petit bruit.
-papa|Tu as entendu le cube ?
-enfant-m|Oui, papa.
-narrateur|Raphaël pose un autre cube.
-narrateur|Jaune encore.
-narrateur|Aniss avance un pied.
-narrateur|Puis il s'assoit au bord.
-narrateur|Il observe d'abord.
-narrateur|Plus tard, il pose un cube.
-narrateur|Tout doux.
-maman|C'est assez.
-papa|Tu as répété, Raphaël.
-papa|Bravo.
-maman|Tu as fait du bon travail.
-enfant-m|Aniss a observé d'abord.
-maman|Oui.
-maman|Il a pu observer d'abord.
-narrateur|Une goutte glisse encore sur la vitre.
-narrateur|Elle va tout droit, puis elle tourne.
-papa|Tu la vois, Raphaël ?
+enfant-m|Aniss.
+enfant-m|Tu viens ?
+narrateur|Aniss ne vient pas encore.
+enfant-m|Le wagon rouge est pour lui.
+narrateur|Raphaël regarde papa.
+papa|On peut répéter, tout doux.
+maman|On peut observer d'abord.
+enfant-m|D'accord.
+narrateur|Le wagon rouge attend par terre.
+narrateur|Il est lisse et froid.
+papa|Tu parles tout bas, d'accord ?
+enfant-m|D'accord, papa.
+narrateur|Une miette est sur le wagon.
+papa|Tu as vu la miette ?
 enfant-m|Oui.
-narrateur|Raphaël attend encore un peu.
-narrateur|Aniss pose sa main près du panier.
-narrateur|Il prend un cube jaune.
-narrateur|Il le tourne.
-narrateur|Le cube est lisse.
-maman|Tu as répété la règle ?
-enfant-m|Un cube.
-enfant-m|Puis on attend.
-papa|Bravo.
-narrateur|Le tapis rouge reste chaud.
-narrateur|Le savon sent encore dans le couloir.</t>
+narrateur|Raphaël souffle.
+narrateur|La miette part.
+maman|Le train peut avancer un peu.
+narrateur|Raphaël pousse le wagon brun.
+narrateur|Aniss regarde, près du buffet.
+narrateur|Ses pieds restent au même endroit.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pluie,manteaux</t>
+          <t>cuisine,bois</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1415,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Estelle a besoin de calme. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>Aniss a besoin de calme. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1515,7 +1494,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.28</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1591,7 +1570,6 @@
 narrateur|Que peut-on faire ?</t>
         </is>
       </c>
-      <c r="AX3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1616,12 +1594,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a su répéter. Aniss a pu observer d'abord. Le jeu a continué, tout doux. Le tapis reste rouge et chaud. Tu as laissé le temps ? Oui, papa. Bravo. Observer d'abord, c'est bien. Aniss touche encore un cube. Il le pose près des autres. Raphaël attend. C'est du bon travail.</t>
+          <t>Raphaël va près du buffet. Il parle tout bas. Un wagon. Puis on attend. C'est répéter, tout doux. Aniss écoute. Il va observer d'abord. Ses mains restent sur le bois. Raphaël pose un wagon bleu. Il attend. Tu as répété, Raphaël ? Oui, papa. Aniss peut regarder. Aniss avance un pied. Puis il s'arrête. Il observe d'abord. C'est bien. Le train a trois wagons. Il manque le rouge. Il attend encore un peu. Raphaël pousse le train. Il passe près du buffet. Aniss suit des yeux.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Adèle a su &lt;emphasis level="moderate"&gt;répéter&lt;/emphasis&gt;. Estelle a pu observer d'abord. Le jeu a continué.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Raphaël va près du buffet. Il parle tout bas. Un wagon. Puis on attend. C'est répéter, tout doux. Aniss écoute. Il va observer d'abord. Ses mains restent sur le bois. Raphaël pose un wagon bleu. Il attend. Tu as répété, Raphaël ? Oui, papa. Aniss peut regarder. Aniss avance un pied. Puis il s'arrête. Il observe d'abord. C'est bien. Le train a trois wagons. Il manque le rouge. Il attend encore un peu. Raphaël pousse le train. Il passe près du buffet. Aniss suit des yeux.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1684,7 +1662,7 @@
         <v>0.86</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1760,21 +1738,36 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a su répéter.
-narrateur|Aniss a pu observer d'abord.
-narrateur|Le jeu a continué, tout doux.
-narrateur|Le tapis reste rouge et chaud.
-papa|Tu as laissé le temps ?
+          <t>narrateur|Raphaël va près du buffet.
+narrateur|Il parle tout bas.
+enfant-m|Un wagon.
+enfant-m|Puis on attend.
+narrateur|C'est répéter, tout doux.
+narrateur|Aniss écoute.
+narrateur|Il va observer d'abord.
+narrateur|Ses mains restent sur le bois.
+narrateur|Raphaël pose un wagon bleu.
+narrateur|Il attend.
+papa|Tu as répété, Raphaël ?
 enfant-m|Oui, papa.
-maman|Bravo.
-maman|Observer d'abord, c'est bien.
-narrateur|Aniss touche encore un cube.
-narrateur|Il le pose près des autres.
-narrateur|Raphaël attend.
-papa|C'est du bon travail.</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr"/>
+maman|Aniss peut regarder.
+narrateur|Aniss avance un pied.
+narrateur|Puis il s'arrête.
+narrateur|Il observe d'abord.
+papa|C'est bien.
+narrateur|Le train a trois wagons.
+enfant-m|Il manque le rouge.
+maman|Il attend encore un peu.
+narrateur|Raphaël pousse le train.
+narrateur|Il passe près du buffet.
+narrateur|Aniss suit des yeux.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>bois</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1799,12 +1792,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range les cubes ? Oui. Raphaël met un cube dans le panier. Aniss met un cube aussi. Le panier redevient lourd. Tu as fini de ranger tes cubes ? Oui, papa. Bravo, Raphaël. Merci, Aniss. Papa tend la main. Le couloir sent encore le savon. Les manteaux sont un peu secs.</t>
+          <t>Plus tard, Aniss tend la main. Il prend le wagon rouge. Il le pose, tout doux. Ça fait clic. Merci, Aniss. Tu as laissé le temps. Bravo, Raphaël. Le train passe sous la table. Il va vers la chaise. Il arrive, papa ? Bientôt. Un pied de chaise est proche. Le train le touche. Il est arrivé. Oui. Jusqu'à la chaise. Raphaël souffle comme un sifflet. Aniss souffle un tout petit peu. Tu as fini ton train ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Papa reprend Adèle. Estelle range un cube.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>Plus tard, Aniss tend la main. Il prend le wagon rouge. Il le pose, tout doux. Ça fait clic. Merci, Aniss. Tu as laissé le temps. Bravo, Raphaël. Le train passe sous la table. Il va vers la chaise. Il arrive, papa ? Bientôt. Un pied de chaise est proche. Le train le touche. Il est arrivé. Oui. Jusqu'à la chaise. Raphaël souffle comme un sifflet. Aniss souffle un tout petit peu. Tu as fini ton train ? Oui, papa.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1867,7 +1860,7 @@
         <v>0.86</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1935,21 +1928,33 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On range les cubes ?
-enfant-m|Oui.
-narrateur|Raphaël met un cube dans le panier.
-narrateur|Aniss met un cube aussi.
-narrateur|Le panier redevient lourd.
-papa|Tu as fini de ranger tes cubes ?
-enfant-m|Oui, papa.
-papa|Bravo, Raphaël.
-maman|Merci, Aniss.
-narrateur|Papa tend la main.
-narrateur|Le couloir sent encore le savon.
-narrateur|Les manteaux sont un peu secs.</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr"/>
+          <t>narrateur|Plus tard, Aniss tend la main.
+narrateur|Il prend le wagon rouge.
+narrateur|Il le pose, tout doux.
+narrateur|Ça fait clic.
+enfant-m|Merci, Aniss.
+papa|Tu as laissé le temps.
+maman|Bravo, Raphaël.
+narrateur|Le train passe sous la table.
+narrateur|Il va vers la chaise.
+enfant-m|Il arrive, papa ?
+papa|Bientôt.
+narrateur|Un pied de chaise est proche.
+narrateur|Le train le touche.
+enfant-m|Il est arrivé.
+maman|Oui.
+maman|Jusqu'à la chaise.
+narrateur|Raphaël souffle comme un sifflet.
+narrateur|Aniss souffle un tout petit peu.
+papa|Tu as fini ton train ?
+enfant-m|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>bois</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1974,12 +1979,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a répété. Aniss a observé d'abord. Bravo. Tu as fait du bon travail. Les cubes jaunes dorment. L'histoire est finie.</t>
+          <t>Le wagon rouge brille encore. On a attendu. Aniss a regardé d'abord. Puis le train a avancé. Oui. La confiture sent encore bon. Une miette reste sur la nappe. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="low"&gt;L'histoire est finie.&lt;/prosody&gt;&lt;break time="600ms"/&gt;&lt;/speak&gt;</t>
+          <t>Le wagon rouge brille encore. On a attendu. Aniss a regardé d'abord. Puis le train a avancé. Oui. La confiture sent encore bon. Une miette reste sur la nappe. L'histoire est finie.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2042,7 +2047,7 @@
         <v>0.82</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.22</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2114,15 +2119,16 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|On a répété.
-enfant-m|Aniss a observé d'abord.
-maman|Bravo.
-papa|Tu as fait du bon travail.
-narrateur|Les cubes jaunes dorment.
+          <t>narrateur|Le wagon rouge brille encore.
+enfant-m|On a attendu.
+enfant-m|Aniss a regardé d'abord.
+maman|Puis le train a avancé.
+papa|Oui.
+narrateur|La confiture sent encore bon.
+narrateur|Une miette reste sur la nappe.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
-      <c r="AX6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -2141,7 +2147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2213,13 @@
       <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-009 ouverture du monde, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-06 Raphaël répète, Aniss observe
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-06.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le train sous la table</t>
+          <t>Raphaël répète, Aniss observe</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, matin, nappe à carreaux</t>
+          <t>classe, tapis, vitre embuée, gouttes, manteaux, couloir</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, Aniss, papa, maman</t>
+          <t>Aniss, Raphaël, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut que son train de bois passe sous la table jusqu'à la chaise. Aniss reste près du buffet. Raphaël répète : un wagon, puis on attend. Aniss observe d'abord, puis pose le wagon rouge. Le train arrive.</t>
+          <t>Une goutte quitte un manteau bleu. Sur le rond, un éclat de couloir brille. Aniss veut le rond, maintenant. Raphaël court, sa voix part trop fort : Aniss recule. Raphaël refuse de foncer, dit les mots plus bas, une seconde fois. Merci vécu. Aniss observe, s'assoit. Ils glissent vers le rond. Un éclat de couloir reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La confiture d'abricot brille dans le pot. Elle est orange et un peu épaisse. Le pain grillé sent encore le four. Une miette colle à la nappe. La nappe a des carreaux rouges. Papa essuie la cuillère de bois. Raphaël, tu veux de la confiture ? Oui, papa. Un peu, s'il te plaît. Maman ouvre le tiroir du bas. Dedans, le train de bois attend. Les wagons sont lisses et froids. Tu as vu le train, Raphaël ? Oui. Il va sous la table. Jusqu'à la chaise ? Oui. Le wagon rouge aussi. En ce moment, Raphaël s'assoit. Le carrelage est un peu froid. Il pose un wagon brun. Ça fait un petit clic. Tu as entendu le clic ? Oui, papa. Maman ouvre la porte. Aniss arrive tout doux. Il reste près du buffet. Ses mains touchent le bois. Il a besoin de calme. Aniss. Tu viens ? Aniss ne vient pas encore. Le wagon rouge est pour lui. Raphaël regarde papa. On peut répéter, tout doux. On peut observer d'abord. D'accord. Le wagon rouge attend par terre. Il est lisse et froid. Tu parles tout bas, d'accord ? D'accord, papa. Une miette est sur le wagon. Tu as vu la miette ? Oui. Raphaël souffle. La miette part. Le train peut avancer un peu. Raphaël pousse le wagon brun. Aniss regarde, près du buffet. Ses pieds restent au même endroit.</t>
+          <t>Une goutte quitte un manteau bleu. Elle tombe dans le couloir. L'eau fait un rond sombre. Sur le rond, un éclat de couloir brille. Aniss se penche vers le rond. Il est petit, papa. Tu le vois, Aniss ? Oui, sur l'eau. Les manteaux gouttent, près de la porte. Ça sent le savon, un peu. Ton manteau va là, Aniss. Maman accroche le manteau bleu. La laine est lourde d'eau. Il goutte, maman. Oui, dans le couloir. Le sol du couloir est froid. Une flaque luit sous les crochets. La vitre de la classe est embuée. Des gouttes y glissent, lentes. Tu vois le jardin, Raphaël ? Raphaël pose le nez sur la vitre. Oui, papa. Maman essuie un coin de vitre. Les arbres sont mouillés. Le jardin est gris, derrière. Le tapis rouge attend, un peu rêche. Raphaël s'avance vers le tapis. Raphaël se tourne vers Aniss. On joue, Aniss ? Aniss reste près du mur. Ses mains restent sur ses genoux. Aniss ouvre la bouche. Je veux le rond, maintenant ! Tu restes près de nous ? Oui, papa. En ce moment, Raphaël court vers Aniss. Raphaël tend la main trop vite. Viens, Aniss ! Sa voix part trop fort, trop vite. Aniss recule contre le mur. Oh. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. L'éclat de couloir tremble, puis tient. Raphaël baisse les bras. Il ne vient pas, maman. Les épaules d'Aniss tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La confiture d'abricot brille dans le pot. Elle est orange et un peu épaisse. Le pain grillé sent encore le four. Une miette colle à la nappe. La nappe a des carreaux rouges. Papa essuie la cuillère de bois. Raphaël, tu veux de la confiture ? Oui, papa. Un peu, s'il te plaît. Maman ouvre le tiroir du bas. Dedans, le train de bois attend. Les wagons sont lisses et froids. Tu as vu le train, Raphaël ? Oui. Il va sous la table. Jusqu'à la chaise ? Oui. Le wagon rouge aussi. En ce moment, Raphaël s'assoit. Le carrelage est un peu froid. Il pose un wagon brun. Ça fait un petit clic. Tu as entendu le clic ? Oui, papa. Maman ouvre la porte. Aniss arrive tout doux. Il reste près du buffet. Ses mains touchent le bois. Il a besoin de calme. Aniss. Tu viens ? Aniss ne vient pas encore. Le wagon rouge est pour lui. Raphaël regarde papa. On peut répéter, tout doux. On peut observer d'abord. D'accord. Le wagon rouge attend par terre. Il est lisse et froid. Tu parles tout bas, d'accord ? D'accord, papa. Une miette est sur le wagon. Tu as vu la miette ? Oui. Raphaël souffle. La miette part. Le train peut avancer un peu. Raphaël pousse le wagon brun. Aniss regarde, près du buffet. Ses pieds restent au même endroit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte quitte un manteau bleu. Elle tombe dans le couloir. L'eau fait un rond sombre. Sur le rond, un &lt;emphasis level="moderate"&gt;éclat de couloir&lt;/emphasis&gt; brille. Aniss se penche vers le rond. Il est petit, papa. Tu le vois, Aniss ? Oui, sur l'eau. Les manteaux gouttent, près de la porte. Ça sent le savon, un peu. Ton manteau va là, Aniss. Maman accroche le manteau bleu. La laine est lourde d'eau. Il goutte, maman. Oui, dans le couloir. Le sol du couloir est froid. Une flaque luit sous les crochets. La vitre de la classe est embuée. Des gouttes y glissent, lentes. Tu vois le jardin, Raphaël ? Raphaël pose le nez sur la vitre. Oui, papa. Maman essuie un coin de vitre. Les arbres sont mouillés. Le jardin est gris, derrière. Le tapis rouge attend, un peu rêche. Raphaël s'avance vers le tapis. Raphaël se tourne vers Aniss. On joue, Aniss ? Aniss reste près du mur. Ses mains restent sur ses genoux. Aniss ouvre la bouche. Je veux le rond, maintenant ! Tu restes près de nous ? Oui, papa. En ce moment, Raphaël court vers Aniss. Raphaël tend la main trop vite. Viens, Aniss ! Sa voix part trop fort, trop vite. Aniss recule contre le mur. Oh. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. L'éclat de couloir tremble, puis tient. Raphaël baisse les bras. Il ne vient pas, maman. Les épaules d'Aniss tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adèle arrive en classe. Papa est à la porte. Un jeu commence. On pose un cube. Puis on attend. Estelle reste près du mur. Elle a besoin de calme. Adèle va vers Estelle. Adèle va &lt;emphasis&gt;répéter&lt;/emphasis&gt; la règle. Adèle dit : un cube, puis on attend. Estelle écoute. Elle va observer d'abord. Observer d'abord, c'est possible. Adèle joue. Estelle regarde. Papa dit : on peut répéter. On peut observer d'abord. Plus tard, Estelle s'assoit. Elle pose un cube. C'est assez.&lt;/slow&gt; [pause]</t>
+          <t>Une goutte quitte un manteau bleu. Elle tombe dans le couloir. L'eau fait un rond sombre. Sur le rond, un &lt;emphasis&gt;éclat de couloir&lt;/emphasis&gt; brille. Aniss se penche vers le rond. Il est petit, papa. Tu le vois, Aniss ? Oui, sur l'eau. Les manteaux gouttent, près de la porte. Ça sent le savon, un peu. Ton manteau va là, Aniss. Maman accroche le manteau bleu. La laine est lourde d'eau. Il goutte, maman. Oui, dans le couloir. Le sol du couloir est froid. Une flaque luit sous les crochets. La vitre de la classe est embuée. Des gouttes y glissent, lentes. Tu vois le jardin, Raphaël ? Raphaël pose le nez sur la vitre. Oui, papa. Maman essuie un coin de vitre. Les arbres sont mouillés. Le jardin est gris, derrière. Le tapis rouge attend, un peu rêche. Raphaël s'avance vers le tapis. Raphaël se tourne vers Aniss. On joue, Aniss ? Aniss reste près du mur. Ses mains restent sur ses genoux. Aniss ouvre la bouche. Je veux le rond, maintenant ! Tu restes près de nous ? Oui, papa. En ce moment, Raphaël court vers Aniss. Raphaël tend la main trop vite. Viens, Aniss ! Sa voix part trop fort, trop vite. Aniss recule contre le mur. Oh. Le sourire d'Aniss disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. L'éclat de couloir tremble, puis tient. Raphaël baisse les bras. Il ne vient pas, maman. Les épaules d'Aniss tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de couloir</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,66 +1324,70 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=aniss_veut_le_rond_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La confiture d'abricot brille dans le pot.
-narrateur|Elle est orange et un peu épaisse.
-narrateur|Le pain grillé sent encore le four.
-narrateur|Une miette colle à la nappe.
-narrateur|La nappe a des carreaux rouges.
-narrateur|Papa essuie la cuillère de bois.
-papa|Raphaël, tu veux de la confiture ?
+          <t>narrateur|Une goutte quitte un manteau bleu.
+narrateur|Elle tombe dans le couloir.
+narrateur|L'eau fait un rond sombre.
+narrateur|Sur le rond, un éclat de couloir brille.
+narrateur|Aniss se penche vers le rond.
+enfant-m|Il est petit, papa.
+papa|Tu le vois, Aniss ?
+enfant-m|Oui, sur l'eau.
+narrateur|Les manteaux gouttent, près de la porte.
+narrateur|Ça sent le savon, un peu.
+maman|Ton manteau va là, Aniss.
+narrateur|Maman accroche le manteau bleu.
+narrateur|La laine est lourde d'eau.
+enfant-m|Il goutte, maman.
+maman|Oui, dans le couloir.
+narrateur|Le sol du couloir est froid.
+narrateur|Une flaque luit sous les crochets.
+narrateur|La vitre de la classe est embuée.
+narrateur|Des gouttes y glissent, lentes.
+papa|Tu vois le jardin, Raphaël ?
+narrateur|Raphaël pose le nez sur la vitre.
 enfant-m|Oui, papa.
-enfant-m|Un peu, s'il te plaît.
-narrateur|Maman ouvre le tiroir du bas.
-narrateur|Dedans, le train de bois attend.
-narrateur|Les wagons sont lisses et froids.
-maman|Tu as vu le train, Raphaël ?
-enfant-m|Oui.
-enfant-m|Il va sous la table.
-maman|Jusqu'à la chaise ?
-enfant-m|Oui.
-enfant-m|Le wagon rouge aussi.
-narrateur|En ce moment, Raphaël s'assoit.
-narrateur|Le carrelage est un peu froid.
-narrateur|Il pose un wagon brun.
-narrateur|Ça fait un petit clic.
-papa|Tu as entendu le clic ?
+narrateur|Maman essuie un coin de vitre.
+maman|Les arbres sont mouillés.
+narrateur|Le jardin est gris, derrière.
+narrateur|Le tapis rouge attend, un peu rêche.
+narrateur|Raphaël s'avance vers le tapis.
+narrateur|Raphaël se tourne vers Aniss.
+enfant-m|On joue, Aniss ?
+narrateur|Aniss reste près du mur.
+narrateur|Ses mains restent sur ses genoux.
+narrateur|Aniss ouvre la bouche.
+enfant-m|Je veux le rond, maintenant !
+papa|Tu restes près de nous ?
 enfant-m|Oui, papa.
-narrateur|Maman ouvre la porte.
-narrateur|Aniss arrive tout doux.
-narrateur|Il reste près du buffet.
-narrateur|Ses mains touchent le bois.
-narrateur|Il a besoin de calme.
-enfant-m|Aniss.
-enfant-m|Tu viens ?
-narrateur|Aniss ne vient pas encore.
-enfant-m|Le wagon rouge est pour lui.
-narrateur|Raphaël regarde papa.
-papa|On peut répéter, tout doux.
-maman|On peut observer d'abord.
-enfant-m|D'accord.
-narrateur|Le wagon rouge attend par terre.
-narrateur|Il est lisse et froid.
-papa|Tu parles tout bas, d'accord ?
-enfant-m|D'accord, papa.
-narrateur|Une miette est sur le wagon.
-papa|Tu as vu la miette ?
-enfant-m|Oui.
-narrateur|Raphaël souffle.
-narrateur|La miette part.
-maman|Le train peut avancer un peu.
-narrateur|Raphaël pousse le wagon brun.
-narrateur|Aniss regarde, près du buffet.
-narrateur|Ses pieds restent au même endroit.</t>
+narrateur|En ce moment, Raphaël court vers Aniss.
+narrateur|Raphaël tend la main trop vite.
+enfant-m|Viens, Aniss !
+narrateur|Sa voix part trop fort, trop vite.
+narrateur|Aniss recule contre le mur.
+enfant-m|Oh.
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|L'éclat de couloir tremble, puis tient.
+narrateur|Raphaël baisse les bras.
+enfant-m|Il ne vient pas, maman.
+narrateur|Les épaules d'Aniss tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>cuisine,bois</t>
+          <t>pluie,manteaux</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Estelle a besoin de calme. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1445,7 +1449,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut répéter. On peut observer d'abord. Que fait-on ?</t>
+          <t>On peut répéter. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1483,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1491,10 +1495,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1509,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1545,13 +1553,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1561,7 +1569,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_dit_les_mots_une_seconde_fois; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1594,17 +1602,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël va près du buffet. Il parle tout bas. Un wagon. Puis on attend. C'est répéter, tout doux. Aniss écoute. Il va observer d'abord. Ses mains restent sur le bois. Raphaël pose un wagon bleu. Il attend. Tu as répété, Raphaël ? Oui, papa. Aniss peut regarder. Aniss avance un pied. Puis il s'arrête. Il observe d'abord. C'est bien. Le train a trois wagons. Il manque le rouge. Il attend encore un peu. Raphaël pousse le train. Il passe près du buffet. Aniss suit des yeux.</t>
+          <t>Raphaël avance trop vite vers Aniss. Viens, Aniss ! Sa voix se mélange au bruit des gouttes. Aniss serre les genoux. Oh. Raphaël refuse de foncer. Il referme la main. Il regarde Aniss, un instant. Tu veux venir près du tapis ? Papa s'accroupit à la même hauteur. Raphaël pose un genou près du tapis. Le tapis est rêche, un peu froid. Viens, Aniss. Il dit les mots plus bas. Viens, Aniss. Papa dit les mots, comme lui. Viens, Aniss. Raphaël dit les mots, une seconde fois. Merci, Raphaël. Maman a entendu toute la phrase. Aniss écoute. Il regarde le tapis. Ses mains restent un moment. Puis il avance un pied. Il s'assoit au bord. Je suis là. Le ventre d'Aniss se desserre. Tu as les mains au chaud ? Un peu, papa. On voit le tapis ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël va près du buffet. Il parle tout bas. Un wagon. Puis on attend. C'est répéter, tout doux. Aniss écoute. Il va observer d'abord. Ses mains restent sur le bois. Raphaël pose un wagon bleu. Il attend. Tu as répété, Raphaël ? Oui, papa. Aniss peut regarder. Aniss avance un pied. Puis il s'arrête. Il observe d'abord. C'est bien. Le train a trois wagons. Il manque le rouge. Il attend encore un peu. Raphaël pousse le train. Il passe près du buffet. Aniss suit des yeux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël avance trop vite vers Aniss. &lt;emphasis level="moderate"&gt;Viens&lt;/emphasis&gt;, Aniss ! Sa voix se mélange au bruit des gouttes. Aniss serre les genoux. Oh. Raphaël refuse de foncer. Il referme la main. Il regarde Aniss, un instant. Tu veux venir près du tapis ? Papa s'accroupit à la même hauteur. Raphaël pose un genou près du tapis. Le tapis est rêche, un peu froid. Viens, Aniss. Il dit les mots plus bas. Viens, Aniss. Papa dit les mots, comme lui. Viens, Aniss. Raphaël dit les mots, une seconde fois. Merci, Raphaël. Maman a entendu toute la phrase. Aniss écoute. Il regarde le tapis. Ses mains restent un moment. Puis il avance un pied. Il s'assoit au bord. Je suis là. Le ventre d'Aniss se desserre. Tu as les mains au chaud ? Un peu, papa. On voit le tapis ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adèle a su &lt;emphasis&gt;répéter&lt;/emphasis&gt;. Estelle a pu observer d'abord. Le jeu a continué.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël avance trop vite vers Aniss. &lt;emphasis&gt;Viens&lt;/emphasis&gt;, Aniss ! Sa voix se mélange au bruit des gouttes. Aniss serre les genoux. Oh. Raphaël refuse de foncer. Il referme la main. Il regarde Aniss, un instant. Tu veux venir près du tapis ? Papa s'accroupit à la même hauteur. Raphaël pose un genou près du tapis. Le tapis est rêche, un peu froid. Viens, Aniss. Il dit les mots plus bas. Viens, Aniss. Papa dit les mots, comme lui. Viens, Aniss. Raphaël dit les mots, une seconde fois. Merci, Raphaël. Maman a entendu toute la phrase. Aniss écoute. Il regarde le tapis. Ses mains restent un moment. Puis il avance un pied. Il s'assoit au bord. Je suis là. Le ventre d'Aniss se desserre. Tu as les mains au chaud ? Un peu, papa. On voit le tapis ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1651,18 +1659,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1685,30 +1693,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>Viens</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1717,10 +1725,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1729,43 +1737,51 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=raphael_dit_les_mots_plus_bas; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël va près du buffet.
-narrateur|Il parle tout bas.
-enfant-m|Un wagon.
-enfant-m|Puis on attend.
-narrateur|C'est répéter, tout doux.
+          <t>narrateur|Raphaël avance trop vite vers Aniss.
+enfant-m|Viens, Aniss !
+narrateur|Sa voix se mélange au bruit des gouttes.
+narrateur|Aniss serre les genoux.
+enfant-m|Oh.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la main.
+narrateur|Il regarde Aniss, un instant.
+papa|Tu veux venir près du tapis ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Raphaël pose un genou près du tapis.
+narrateur|Le tapis est rêche, un peu froid.
+enfant-m|Viens, Aniss.
+narrateur|Il dit les mots plus bas.
+papa|Viens, Aniss.
+narrateur|Papa dit les mots, comme lui.
+enfant-m|Viens, Aniss.
+narrateur|Raphaël dit les mots, une seconde fois.
+maman|Merci, Raphaël.
+narrateur|Maman a entendu toute la phrase.
 narrateur|Aniss écoute.
-narrateur|Il va observer d'abord.
-narrateur|Ses mains restent sur le bois.
-narrateur|Raphaël pose un wagon bleu.
-narrateur|Il attend.
-papa|Tu as répété, Raphaël ?
-enfant-m|Oui, papa.
-maman|Aniss peut regarder.
-narrateur|Aniss avance un pied.
-narrateur|Puis il s'arrête.
-narrateur|Il observe d'abord.
-papa|C'est bien.
-narrateur|Le train a trois wagons.
-enfant-m|Il manque le rouge.
-maman|Il attend encore un peu.
-narrateur|Raphaël pousse le train.
-narrateur|Il passe près du buffet.
-narrateur|Aniss suit des yeux.</t>
+narrateur|Il regarde le tapis.
+narrateur|Ses mains restent un moment.
+narrateur|Puis il avance un pied.
+narrateur|Il s'assoit au bord.
+enfant-m|Je suis là.
+narrateur|Le ventre d'Aniss se desserre.
+papa|Tu as les mains au chaud ?
+enfant-m|Un peu, papa.
+maman|On voit le tapis ?
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>bois</t>
+          <t>tapis,gouttes</t>
         </is>
       </c>
     </row>
@@ -1792,17 +1808,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Aniss tend la main. Il prend le wagon rouge. Il le pose, tout doux. Ça fait clic. Merci, Aniss. Tu as laissé le temps. Bravo, Raphaël. Le train passe sous la table. Il va vers la chaise. Il arrive, papa ? Bientôt. Un pied de chaise est proche. Le train le touche. Il est arrivé. Oui. Jusqu'à la chaise. Raphaël souffle comme un sifflet. Aniss souffle un tout petit peu. Tu as fini ton train ? Oui, papa.</t>
+          <t>Raphaël tire Aniss trop vite. Le rond, maintenant ! Le pied d'Aniss glisse sur l'eau. Oh. Un manteau bouge, puis retombe. Aniss avance la main. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Aniss observe le couloir. Il écoute les gouttes. Sur le rond, un éclat de couloir luit. Là, près du manteau bleu. Aniss tient la manche de Raphaël. La laine est froide, un peu lourde. Elle est froide, papa. Tu marches jusqu'au rond ? Oui, papa. On avance ? Oui, maman. Ils posent un pied, puis l'autre. Le sol mouillé touche les chaussettes. L'air froid revient sur les joues. Je le tiens. On marche. Aniss serre la manche contre lui. Je la tiens. On avance. Ils passent le long des manteaux. La laine gratte, un peu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Aniss tend la main. Il prend le wagon rouge. Il le pose, tout doux. Ça fait clic. Merci, Aniss. Tu as laissé le temps. Bravo, Raphaël. Le train passe sous la table. Il va vers la chaise. Il arrive, papa ? Bientôt. Un pied de chaise est proche. Le train le touche. Il est arrivé. Oui. Jusqu'à la chaise. Raphaël souffle comme un sifflet. Aniss souffle un tout petit peu. Tu as fini ton train ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël tire Aniss trop vite. Le rond, maintenant ! Le pied d'Aniss glisse sur l'eau. Oh. Un manteau bouge, puis retombe. Aniss avance la main. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Aniss observe le couloir. Il écoute les gouttes. Sur le rond, un &lt;emphasis level="moderate"&gt;éclat de couloir&lt;/emphasis&gt; luit. Là, près du manteau bleu. Aniss tient la manche de Raphaël. La laine est froide, un peu lourde. Elle est froide, papa. Tu marches jusqu'au rond ? Oui, papa. On avance ? Oui, maman. Ils posent un pied, puis l'autre. Le sol mouillé touche les chaussettes. L'air froid revient sur les joues. Je le tiens. On marche. Aniss serre la manche contre lui. Je la tiens. On avance. Ils passent le long des manteaux. La laine gratte, un peu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Papa reprend Adèle. Estelle range un cube.&lt;/slow&gt; [pause]</t>
+          <t>Raphaël tire Aniss trop vite. Le rond, maintenant ! Le pied d'Aniss glisse sur l'eau. Oh. Un manteau bouge, puis retombe. Aniss avance la main. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Aniss observe le couloir. Il écoute les gouttes. Sur le rond, un &lt;emphasis&gt;éclat de couloir&lt;/emphasis&gt; luit. Là, près du manteau bleu. Aniss tient la manche de Raphaël. La laine est froide, un peu lourde. Elle est froide, papa. Tu marches jusqu'au rond ? Oui, papa. On avance ? Oui, maman. Ils posent un pied, puis l'autre. Le sol mouillé touche les chaussettes. L'air froid revient sur les joues. Je le tiens. On marche. Aniss serre la manche contre lui. Je la tiens. On avance. Ils passent le long des manteaux. La laine gratte, un peu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1849,18 +1865,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1881,28 +1897,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de couloir</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1911,10 +1931,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1923,36 +1943,50 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=aniss_refuse_de_glisser_sans_regarder; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Aniss tend la main.
-narrateur|Il prend le wagon rouge.
-narrateur|Il le pose, tout doux.
-narrateur|Ça fait clic.
-enfant-m|Merci, Aniss.
-papa|Tu as laissé le temps.
-maman|Bravo, Raphaël.
-narrateur|Le train passe sous la table.
-narrateur|Il va vers la chaise.
-enfant-m|Il arrive, papa ?
-papa|Bientôt.
-narrateur|Un pied de chaise est proche.
-narrateur|Le train le touche.
-enfant-m|Il est arrivé.
-maman|Oui.
-maman|Jusqu'à la chaise.
-narrateur|Raphaël souffle comme un sifflet.
-narrateur|Aniss souffle un tout petit peu.
-papa|Tu as fini ton train ?
-enfant-m|Oui, papa.</t>
+          <t>narrateur|Raphaël tire Aniss trop vite.
+enfant-m|Le rond, maintenant !
+narrateur|Le pied d'Aniss glisse sur l'eau.
+enfant-m|Oh.
+narrateur|Un manteau bouge, puis retombe.
+narrateur|Aniss avance la main.
+narrateur|Puis il s'arrête net.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Aniss observe le couloir.
+narrateur|Il écoute les gouttes.
+narrateur|Sur le rond, un éclat de couloir luit.
+enfant-m|Là, près du manteau bleu.
+narrateur|Aniss tient la manche de Raphaël.
+narrateur|La laine est froide, un peu lourde.
+enfant-m|Elle est froide, papa.
+papa|Tu marches jusqu'au rond ?
+enfant-m|Oui, papa.
+maman|On avance ?
+enfant-m|Oui, maman.
+narrateur|Ils posent un pied, puis l'autre.
+narrateur|Le sol mouillé touche les chaussettes.
+narrateur|L'air froid revient sur les joues.
+enfant-m|Je le tiens.
+papa|On marche.
+narrateur|Aniss serre la manche contre lui.
+enfant-m|Je la tiens.
+maman|On avance.
+narrateur|Ils passent le long des manteaux.
+narrateur|La laine gratte, un peu.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>bois</t>
+          <t>couloir,manteaux</t>
         </is>
       </c>
     </row>
@@ -1979,17 +2013,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le wagon rouge brille encore. On a attendu. Aniss a regardé d'abord. Puis le train a avancé. Oui. La confiture sent encore bon. Une miette reste sur la nappe.</t>
+          <t>Le rond brillait, papa. Tu le vois, comme dans le couloir ? Oui, un peu pâle. Aniss pose le genou près de l'eau. On le garde près de nous ? Oui, maman. Raphaël s'assoit près du rond. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur l'eau. On est bien, ici. Une goutte quitte le manteau bleu. Elle tombe dans le même rond. On le voit, maman. Tu le vois sur l'eau ? Oui, l'éclat. Le soir reste dans l'air. Un éclat de couloir reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le wagon rouge brille encore. On a attendu. Aniss a regardé d'abord. Puis le train a avancé. Oui. La confiture sent encore bon. Une miette reste sur la nappe.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rond brillait, papa. Tu le vois, comme dans le couloir ? Oui, un peu pâle. Aniss pose le genou près de l'eau. On le garde près de nous ? Oui, maman. Raphaël s'assoit près du rond. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur l'eau. On est bien, ici. Une goutte quitte le manteau bleu. Elle tombe dans le même rond. On le voit, maman. Tu le vois sur l'eau ? Oui, l'éclat. Le soir reste dans l'air. Un &lt;emphasis level="moderate"&gt;éclat de couloir&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rond brillait, papa. Tu le vois, comme dans le couloir ? Oui, un peu pâle. Aniss pose le genou près de l'eau. On le garde près de nous ? Oui, maman. Raphaël s'assoit près du rond. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur l'eau. On est bien, ici. Une goutte quitte le manteau bleu. Elle tombe dans le même rond. On le voit, maman. Tu le vois sur l'eau ? Oui, l'éclat. Le soir reste dans l'air. Un &lt;emphasis&gt;éclat de couloir&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2036,7 +2070,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2044,10 +2078,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2056,12 +2090,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2070,17 +2104,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de couloir</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2089,11 +2127,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2102,30 +2140,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le wagon rouge brille encore.
-enfant-m|On a attendu.
-enfant-m|Aniss a regardé d'abord.
-maman|Puis le train a avancé.
-papa|Oui.
-narrateur|La confiture sent encore bon.
-narrateur|Une miette reste sur la nappe.</t>
+          <t>enfant-m|Le rond brillait, papa.
+papa|Tu le vois, comme dans le couloir ?
+enfant-m|Oui, un peu pâle.
+narrateur|Aniss pose le genou près de l'eau.
+maman|On le garde près de nous ?
+enfant-m|Oui, maman.
+narrateur|Raphaël s'assoit près du rond.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur l'eau.
+maman|On est bien, ici.
+narrateur|Une goutte quitte le manteau bleu.
+narrateur|Elle tombe dans le même rond.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur l'eau ?
+enfant-m|Oui, l'éclat.
+narrateur|Le soir reste dans l'air.
+narrateur|Un éclat de couloir reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>couloir</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2224,6 +2282,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>